<commit_message>
Add Isabella Perry to the current team, italicize scientific names in bios
Moved her photo from docs/www/team/ (built output) to the actual
source folder www/team/ and resized it (was full camera resolution).
Also extends the existing "(Genus species)" italics helper to team
bios, not just the homepage - Isabella's bio has two.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/team.xlsx
+++ b/data/team.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/63ed0a4e98b474dd/Documents/WESOke_Website/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="15" documentId="11_649064B9B696ADEF6B7F9790E2358A36B82AF7B5" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{6D1125CE-1F64-47E4-B25F-6A309EDA8248}"/>
+  <xr:revisionPtr revIDLastSave="20" documentId="11_649064B9B696ADEF6B7F9790E2358A36B82AF7B5" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{137CEA24-6864-4735-BD11-478FF4E4E7CB}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="15">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="20" uniqueCount="18">
   <si>
     <t>name</t>
   </si>
@@ -88,6 +88,15 @@
   </si>
   <si>
     <t>Reese worked as a research technician on the Coastal Western Screech-Owl Project in 2026, supporting ARU set-up and retrieval, trapping and tagging, and other field-related tasks. Reese completed her BSc Honours in Biology at the University of British Columbia Okanagan and is now pursuing an MSc through the University of Northern British Columbia, looking at wolf denning ecology.</t>
+  </si>
+  <si>
+    <t>Isabella Perry</t>
+  </si>
+  <si>
+    <t>issyperry_bio</t>
+  </si>
+  <si>
+    <t>Isabella is a MSc student in the Quantitative Ecology Lab supervised by Dr. Michael Noonan at the University of British Columbia’s Okanagan Campus. Isabella is passionate about connecting behavioral studies to conservation action, with her core research focusing on linking health to habitat use and selection for giant anteaters (Myrmecophaga tridactyla) in the Brazilian Cerrado. Her work with the project involves evaluating how effectively ARUs model habitat occupancy for coastal western screech-owls (Megascops kennicottii) by comparing results for acoustic data against those of GPS tracking data.</t>
   </si>
 </sst>
 </file>
@@ -159,6 +168,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -448,7 +461,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D4"/>
+  <dimension ref="A1:D5"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="18.5703125" customWidth="1"/>
@@ -513,6 +526,20 @@
         <v>14</v>
       </c>
     </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>15</v>
+      </c>
+      <c r="B5" t="s">
+        <v>5</v>
+      </c>
+      <c r="C5" t="s">
+        <v>16</v>
+      </c>
+      <c r="D5" t="s">
+        <v>17</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>